<commit_message>
feat(io-model): multiplicador de emprego e taxa CAT por trabalhador
Adiciona ao 02_io_model.py:
- coef_emprego_e:    e_j = Ocupações_j / X_j
- multiplicador_emprego_me: m_e = e' L (Type I)
- intensidade_per_trab_a_tilde: ã_j = CAT_j / Ocupações_j
- pegada_per_trab_f_tilde:      f̃ = ã' L

A normalização per-trabalhador desfaz o viés de a_j a favor de setores
trabalho-intensivos com baixo VBP, permitindo o exercício clássico de
robustez "ranking f vs ranking f̃" pedido no programa da disciplina
PECO-5054 (item 2.4).
</commit_message>
<xml_diff>
--- a/outputs/tables/resultados_principais.xlsx
+++ b/outputs/tables/resultados_principais.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P36"/>
+  <dimension ref="A1:T36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -509,6 +509,26 @@
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
+          <t>intensidade_per_trab_a_tilde</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>pegada_per_trab_f_tilde</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>coef_emprego_e</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>multiplicador_emprego_me</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
           <t>quadrante</t>
         </is>
       </c>
@@ -563,7 +583,19 @@
       <c r="O2" t="n">
         <v>1.246031058272278</v>
       </c>
-      <c r="P2" t="inlineStr">
+      <c r="P2" t="n">
+        <v>0.0005878657784854562</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>0.006391502920638499</v>
+      </c>
+      <c r="R2" t="n">
+        <v>82.49810858522174</v>
+      </c>
+      <c r="S2" t="n">
+        <v>84.82311090216284</v>
+      </c>
+      <c r="T2" t="inlineStr">
         <is>
           <t>Residual</t>
         </is>
@@ -619,7 +651,19 @@
       <c r="O3" t="n">
         <v>1.366050520830156</v>
       </c>
-      <c r="P3" t="inlineStr">
+      <c r="P3" t="n">
+        <v>0.001060257996112387</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>0.005360264342345386</v>
+      </c>
+      <c r="R3" t="n">
+        <v>23.61809278254902</v>
+      </c>
+      <c r="S3" t="n">
+        <v>29.01393867349796</v>
+      </c>
+      <c r="T3" t="inlineStr">
         <is>
           <t>Residual</t>
         </is>
@@ -675,7 +719,19 @@
       <c r="O4" t="n">
         <v>1.417678421250367</v>
       </c>
-      <c r="P4" t="inlineStr">
+      <c r="P4" t="n">
+        <v>0.002077939773811146</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>0.006096619865605662</v>
+      </c>
+      <c r="R4" t="n">
+        <v>59.18548387096774</v>
+      </c>
+      <c r="S4" t="n">
+        <v>68.37295943428538</v>
+      </c>
+      <c r="T4" t="inlineStr">
         <is>
           <t>Setor-chave de risco</t>
         </is>
@@ -731,7 +787,19 @@
       <c r="O5" t="n">
         <v>1.252553442658074</v>
       </c>
-      <c r="P5" t="inlineStr">
+      <c r="P5" t="n">
+        <v>0.0144173007609131</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>0.01716149470540424</v>
+      </c>
+      <c r="R5" t="n">
+        <v>7.531633160903072</v>
+      </c>
+      <c r="S5" t="n">
+        <v>10.38525547194706</v>
+      </c>
+      <c r="T5" t="inlineStr">
         <is>
           <t>Risco localizado</t>
         </is>
@@ -787,7 +855,19 @@
       <c r="O6" t="n">
         <v>1.532981987987106</v>
       </c>
-      <c r="P6" t="inlineStr">
+      <c r="P6" t="n">
+        <v>0.01711136890951276</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>0.02268590336757088</v>
+      </c>
+      <c r="R6" t="n">
+        <v>0.2742932057541114</v>
+      </c>
+      <c r="S6" t="n">
+        <v>6.309852753541876</v>
+      </c>
+      <c r="T6" t="inlineStr">
         <is>
           <t>Propagador estrutural</t>
         </is>
@@ -843,7 +923,19 @@
       <c r="O7" t="n">
         <v>1.826148968703927</v>
       </c>
-      <c r="P7" t="inlineStr">
+      <c r="P7" t="n">
+        <v>0.0270516717325228</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>0.03630120691174878</v>
+      </c>
+      <c r="R7" t="n">
+        <v>0.4040215494533429</v>
+      </c>
+      <c r="S7" t="n">
+        <v>10.09312743364347</v>
+      </c>
+      <c r="T7" t="inlineStr">
         <is>
           <t>Propagador estrutural</t>
         </is>
@@ -899,7 +991,19 @@
       <c r="O8" t="n">
         <v>1.757645958465375</v>
       </c>
-      <c r="P8" t="inlineStr">
+      <c r="P8" t="n">
+        <v>0.01926935694493104</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>0.02656066880563825</v>
+      </c>
+      <c r="R8" t="n">
+        <v>4.105374370078637</v>
+      </c>
+      <c r="S8" t="n">
+        <v>18.8154195895456</v>
+      </c>
+      <c r="T8" t="inlineStr">
         <is>
           <t>Propagador estrutural</t>
         </is>
@@ -955,7 +1059,19 @@
       <c r="O9" t="n">
         <v>1.353263134232178</v>
       </c>
-      <c r="P9" t="inlineStr">
+      <c r="P9" t="n">
+        <v>0.002683490821890433</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>0.006555518787417437</v>
+      </c>
+      <c r="R9" t="n">
+        <v>27.22898496649721</v>
+      </c>
+      <c r="S9" t="n">
+        <v>31.65738196436137</v>
+      </c>
+      <c r="T9" t="inlineStr">
         <is>
           <t>Residual</t>
         </is>
@@ -1011,7 +1127,19 @@
       <c r="O10" t="n">
         <v>1.383058282476874</v>
       </c>
-      <c r="P10" t="inlineStr">
+      <c r="P10" t="n">
+        <v>0.01443453694711751</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>0.02027328565094768</v>
+      </c>
+      <c r="R10" t="n">
+        <v>15.20698659470635</v>
+      </c>
+      <c r="S10" t="n">
+        <v>19.41158225459135</v>
+      </c>
+      <c r="T10" t="inlineStr">
         <is>
           <t>Risco localizado</t>
         </is>
@@ -1067,7 +1195,19 @@
       <c r="O11" t="n">
         <v>1.439897662971887</v>
       </c>
-      <c r="P11" t="inlineStr">
+      <c r="P11" t="n">
+        <v>0.04512448132780083</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>0.05636768608504349</v>
+      </c>
+      <c r="R11" t="n">
+        <v>0.4210204505006169</v>
+      </c>
+      <c r="S11" t="n">
+        <v>3.916026897057982</v>
+      </c>
+      <c r="T11" t="inlineStr">
         <is>
           <t>Propagador estrutural</t>
         </is>
@@ -1123,7 +1263,19 @@
       <c r="O12" t="n">
         <v>1.693340590279087</v>
       </c>
-      <c r="P12" t="inlineStr">
+      <c r="P12" t="n">
+        <v>0.1082474226804124</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>0.1127137326561248</v>
+      </c>
+      <c r="R12" t="n">
+        <v>2.952636064775356</v>
+      </c>
+      <c r="S12" t="n">
+        <v>41.84858153879676</v>
+      </c>
+      <c r="T12" t="inlineStr">
         <is>
           <t>Setor-chave de risco</t>
         </is>
@@ -1179,7 +1331,19 @@
       <c r="O13" t="n">
         <v>1.44470422662341</v>
       </c>
-      <c r="P13" t="inlineStr">
+      <c r="P13" t="n">
+        <v>0.03068530514831231</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>0.03794360333832337</v>
+      </c>
+      <c r="R13" t="n">
+        <v>2.682949140139041</v>
+      </c>
+      <c r="S13" t="n">
+        <v>6.769993500137541</v>
+      </c>
+      <c r="T13" t="inlineStr">
         <is>
           <t>Propagador estrutural</t>
         </is>
@@ -1235,7 +1399,19 @@
       <c r="O14" t="n">
         <v>1.548205750227505</v>
       </c>
-      <c r="P14" t="inlineStr">
+      <c r="P14" t="n">
+        <v>0.01780630756349428</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>0.02650596049991481</v>
+      </c>
+      <c r="R14" t="n">
+        <v>5.908046848849308</v>
+      </c>
+      <c r="S14" t="n">
+        <v>10.44745027781959</v>
+      </c>
+      <c r="T14" t="inlineStr">
         <is>
           <t>Setor-chave de risco</t>
         </is>
@@ -1291,7 +1467,19 @@
       <c r="O15" t="n">
         <v>1.809772994471501</v>
       </c>
-      <c r="P15" t="inlineStr">
+      <c r="P15" t="n">
+        <v>0.01261686484523918</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>0.0230070074879416</v>
+      </c>
+      <c r="R15" t="n">
+        <v>0.9681223505592385</v>
+      </c>
+      <c r="S15" t="n">
+        <v>7.798715760833368</v>
+      </c>
+      <c r="T15" t="inlineStr">
         <is>
           <t>Propagador estrutural</t>
         </is>
@@ -1347,7 +1535,19 @@
       <c r="O16" t="n">
         <v>1.395621848007814</v>
       </c>
-      <c r="P16" t="inlineStr">
+      <c r="P16" t="n">
+        <v>0.01233337913975539</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>0.01721330832998528</v>
+      </c>
+      <c r="R16" t="n">
+        <v>6.381653950714725</v>
+      </c>
+      <c r="S16" t="n">
+        <v>9.525583530756542</v>
+      </c>
+      <c r="T16" t="inlineStr">
         <is>
           <t>Residual</t>
         </is>
@@ -1403,7 +1603,19 @@
       <c r="O17" t="n">
         <v>1.462474166737531</v>
       </c>
-      <c r="P17" t="inlineStr">
+      <c r="P17" t="n">
+        <v>0.03953229398663697</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>0.04736261633786414</v>
+      </c>
+      <c r="R17" t="n">
+        <v>3.717387479689942</v>
+      </c>
+      <c r="S17" t="n">
+        <v>7.494530347240168</v>
+      </c>
+      <c r="T17" t="inlineStr">
         <is>
           <t>Setor-chave de risco</t>
         </is>
@@ -1459,7 +1671,19 @@
       <c r="O18" t="n">
         <v>1.524433462368046</v>
       </c>
-      <c r="P18" t="inlineStr">
+      <c r="P18" t="n">
+        <v>0.03782692645251887</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>0.05288954389510896</v>
+      </c>
+      <c r="R18" t="n">
+        <v>1.877397413759013</v>
+      </c>
+      <c r="S18" t="n">
+        <v>3.981831731148973</v>
+      </c>
+      <c r="T18" t="inlineStr">
         <is>
           <t>Propagador estrutural</t>
         </is>
@@ -1515,7 +1739,19 @@
       <c r="O19" t="n">
         <v>1.546072200659886</v>
       </c>
-      <c r="P19" t="inlineStr">
+      <c r="P19" t="n">
+        <v>0.004942510511035904</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>0.01089956152577315</v>
+      </c>
+      <c r="R19" t="n">
+        <v>16.00153626226341</v>
+      </c>
+      <c r="S19" t="n">
+        <v>20.86707476518447</v>
+      </c>
+      <c r="T19" t="inlineStr">
         <is>
           <t>Propagador estrutural</t>
         </is>
@@ -1571,7 +1807,19 @@
       <c r="O20" t="n">
         <v>1.395310222104528</v>
       </c>
-      <c r="P20" t="inlineStr">
+      <c r="P20" t="n">
+        <v>0.005763194723668995</v>
+      </c>
+      <c r="Q20" t="n">
+        <v>0.01064947238366128</v>
+      </c>
+      <c r="R20" t="n">
+        <v>13.29028740962655</v>
+      </c>
+      <c r="S20" t="n">
+        <v>16.40812712196992</v>
+      </c>
+      <c r="T20" t="inlineStr">
         <is>
           <t>Residual</t>
         </is>
@@ -1627,7 +1875,19 @@
       <c r="O21" t="n">
         <v>1.359030643753097</v>
       </c>
-      <c r="P21" t="inlineStr">
+      <c r="P21" t="n">
+        <v>0.006664328305857594</v>
+      </c>
+      <c r="Q21" t="n">
+        <v>0.01087461371640277</v>
+      </c>
+      <c r="R21" t="n">
+        <v>7.879692946871963</v>
+      </c>
+      <c r="S21" t="n">
+        <v>11.98150767664957</v>
+      </c>
+      <c r="T21" t="inlineStr">
         <is>
           <t>Residual</t>
         </is>
@@ -1683,7 +1943,19 @@
       <c r="O22" t="n">
         <v>1.486938393116037</v>
       </c>
-      <c r="P22" t="inlineStr">
+      <c r="P22" t="n">
+        <v>0.01890709899721695</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>0.02585607953639441</v>
+      </c>
+      <c r="R22" t="n">
+        <v>8.163007731363951</v>
+      </c>
+      <c r="S22" t="n">
+        <v>14.13026041191768</v>
+      </c>
+      <c r="T22" t="inlineStr">
         <is>
           <t>Setor-chave de risco</t>
         </is>
@@ -1739,7 +2011,19 @@
       <c r="O23" t="n">
         <v>1.324985316106087</v>
       </c>
-      <c r="P23" t="inlineStr">
+      <c r="P23" t="n">
+        <v>0.003291247922330952</v>
+      </c>
+      <c r="Q23" t="n">
+        <v>0.007381090052400618</v>
+      </c>
+      <c r="R23" t="n">
+        <v>20.70049035692151</v>
+      </c>
+      <c r="S23" t="n">
+        <v>25.34963639837747</v>
+      </c>
+      <c r="T23" t="inlineStr">
         <is>
           <t>Residual</t>
         </is>
@@ -1795,7 +2079,19 @@
       <c r="O24" t="n">
         <v>1.578869204487869</v>
       </c>
-      <c r="P24" t="inlineStr">
+      <c r="P24" t="n">
+        <v>0.005518261463192627</v>
+      </c>
+      <c r="Q24" t="n">
+        <v>0.01055396002705657</v>
+      </c>
+      <c r="R24" t="n">
+        <v>4.8841344818005</v>
+      </c>
+      <c r="S24" t="n">
+        <v>11.52915415904947</v>
+      </c>
+      <c r="T24" t="inlineStr">
         <is>
           <t>Propagador estrutural</t>
         </is>
@@ -1851,7 +2147,19 @@
       <c r="O25" t="n">
         <v>1.396887337062903</v>
       </c>
-      <c r="P25" t="inlineStr">
+      <c r="P25" t="n">
+        <v>0.005158668125683915</v>
+      </c>
+      <c r="Q25" t="n">
+        <v>0.008239281946730594</v>
+      </c>
+      <c r="R25" t="n">
+        <v>3.741599387025769</v>
+      </c>
+      <c r="S25" t="n">
+        <v>6.403442756565267</v>
+      </c>
+      <c r="T25" t="inlineStr">
         <is>
           <t>Residual</t>
         </is>
@@ -1907,7 +2215,19 @@
       <c r="O26" t="n">
         <v>1.071845670018026</v>
       </c>
-      <c r="P26" t="inlineStr">
+      <c r="P26" t="n">
+        <v>0.002340745694699883</v>
+      </c>
+      <c r="Q26" t="n">
+        <v>0.003448628816328029</v>
+      </c>
+      <c r="R26" t="n">
+        <v>0.5779983725977939</v>
+      </c>
+      <c r="S26" t="n">
+        <v>1.232842443783011</v>
+      </c>
+      <c r="T26" t="inlineStr">
         <is>
           <t>Residual</t>
         </is>
@@ -1963,7 +2283,19 @@
       <c r="O27" t="n">
         <v>1.319166343156384</v>
       </c>
-      <c r="P27" t="inlineStr">
+      <c r="P27" t="n">
+        <v>0.001858349877649014</v>
+      </c>
+      <c r="Q27" t="n">
+        <v>0.005806421235991065</v>
+      </c>
+      <c r="R27" t="n">
+        <v>22.95273066386898</v>
+      </c>
+      <c r="S27" t="n">
+        <v>26.27467111891976</v>
+      </c>
+      <c r="T27" t="inlineStr">
         <is>
           <t>Residual</t>
         </is>
@@ -2019,7 +2351,19 @@
       <c r="O28" t="n">
         <v>1.233631399664471</v>
       </c>
-      <c r="P28" t="inlineStr">
+      <c r="P28" t="n">
+        <v>0.01535512316687434</v>
+      </c>
+      <c r="Q28" t="n">
+        <v>0.01948977629823254</v>
+      </c>
+      <c r="R28" t="n">
+        <v>10.14804295385573</v>
+      </c>
+      <c r="S28" t="n">
+        <v>12.55220791036853</v>
+      </c>
+      <c r="T28" t="inlineStr">
         <is>
           <t>Risco localizado</t>
         </is>
@@ -2075,7 +2419,19 @@
       <c r="O29" t="n">
         <v>1.1874040841719</v>
       </c>
-      <c r="P29" t="inlineStr">
+      <c r="P29" t="n">
+        <v>0.005307147481802665</v>
+      </c>
+      <c r="Q29" t="n">
+        <v>0.007391215790826917</v>
+      </c>
+      <c r="R29" t="n">
+        <v>8.580372496816176</v>
+      </c>
+      <c r="S29" t="n">
+        <v>10.20347862168812</v>
+      </c>
+      <c r="T29" t="inlineStr">
         <is>
           <t>Residual</t>
         </is>
@@ -2129,7 +2485,19 @@
       <c r="O30" t="n">
         <v>1.206621723887114</v>
       </c>
-      <c r="P30" t="inlineStr">
+      <c r="P30" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q30" t="n">
+        <v>0.00287985481110607</v>
+      </c>
+      <c r="R30" t="n">
+        <v>14.3349176689947</v>
+      </c>
+      <c r="S30" t="n">
+        <v>16.52088504648927</v>
+      </c>
+      <c r="T30" t="inlineStr">
         <is>
           <t>Residual</t>
         </is>
@@ -2185,7 +2553,19 @@
       <c r="O31" t="n">
         <v>1.315884599407887</v>
       </c>
-      <c r="P31" t="inlineStr">
+      <c r="P31" t="n">
+        <v>0.003965321905324861</v>
+      </c>
+      <c r="Q31" t="n">
+        <v>0.008168895173100838</v>
+      </c>
+      <c r="R31" t="n">
+        <v>25.87169291940664</v>
+      </c>
+      <c r="S31" t="n">
+        <v>28.29142638305526</v>
+      </c>
+      <c r="T31" t="inlineStr">
         <is>
           <t>Risco localizado</t>
         </is>
@@ -2239,7 +2619,19 @@
       <c r="O32" t="n">
         <v>1.341763572139528</v>
       </c>
-      <c r="P32" t="inlineStr">
+      <c r="P32" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q32" t="n">
+        <v>0.004117712683728947</v>
+      </c>
+      <c r="R32" t="n">
+        <v>13.29500443393438</v>
+      </c>
+      <c r="S32" t="n">
+        <v>17.52946479987962</v>
+      </c>
+      <c r="T32" t="inlineStr">
         <is>
           <t>Residual</t>
         </is>
@@ -2295,7 +2687,19 @@
       <c r="O33" t="n">
         <v>1.33768544857563</v>
       </c>
-      <c r="P33" t="inlineStr">
+      <c r="P33" t="n">
+        <v>0.04766066290099116</v>
+      </c>
+      <c r="Q33" t="n">
+        <v>0.05564927430340993</v>
+      </c>
+      <c r="R33" t="n">
+        <v>13.60375563983901</v>
+      </c>
+      <c r="S33" t="n">
+        <v>17.51604365456561</v>
+      </c>
+      <c r="T33" t="inlineStr">
         <is>
           <t>Risco localizado</t>
         </is>
@@ -2351,7 +2755,19 @@
       <c r="O34" t="n">
         <v>1.222595804741433</v>
       </c>
-      <c r="P34" t="inlineStr">
+      <c r="P34" t="n">
+        <v>0.004801920768307323</v>
+      </c>
+      <c r="Q34" t="n">
+        <v>0.007370290217398877</v>
+      </c>
+      <c r="R34" t="n">
+        <v>9.887347044478494</v>
+      </c>
+      <c r="S34" t="n">
+        <v>12.17416343607444</v>
+      </c>
+      <c r="T34" t="inlineStr">
         <is>
           <t>Residual</t>
         </is>
@@ -2407,7 +2823,19 @@
       <c r="O35" t="n">
         <v>1.589698338169979</v>
       </c>
-      <c r="P35" t="inlineStr">
+      <c r="P35" t="n">
+        <v>0.00232237007280944</v>
+      </c>
+      <c r="Q35" t="n">
+        <v>0.00772098974511053</v>
+      </c>
+      <c r="R35" t="n">
+        <v>48.05279413184056</v>
+      </c>
+      <c r="S35" t="n">
+        <v>56.69601548430369</v>
+      </c>
+      <c r="T35" t="inlineStr">
         <is>
           <t>Setor-chave de risco</t>
         </is>
@@ -2461,7 +2889,19 @@
       <c r="O36" t="n">
         <v>1</v>
       </c>
-      <c r="P36" t="inlineStr">
+      <c r="P36" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q36" t="n">
+        <v>0</v>
+      </c>
+      <c r="R36" t="n">
+        <v>111.8241055131401</v>
+      </c>
+      <c r="S36" t="n">
+        <v>111.8241055131401</v>
+      </c>
+      <c r="T36" t="inlineStr">
         <is>
           <t>Residual</t>
         </is>

</xml_diff>

<commit_message>
chore(outputs): regenera artefatos com pipeline completo (etapas 1-5)
Atualiza PDF de sensibilidade e XLSX de resultados principais gerados
pela execução completa do pipeline após integração do XLSX oficial IJSN
e do vetor satélite AEAT-2015 real.

https://claude.ai/code/session_01LQ6h1ri8knHdK2ogHrBTYZ
</commit_message>
<xml_diff>
--- a/outputs/tables/resultados_principais.xlsx
+++ b/outputs/tables/resultados_principais.xlsx
@@ -20,16 +20,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -40,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -48,21 +45,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -432,102 +420,102 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>codigo</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>nome</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>vbp_milhoes_RS</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>ocupacoes</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>producao_X</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>demanda_final_Y</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>acidentes_CAT</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>intensidade_direta_a</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>pegada_estrutural_f</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>indireto_f_minus_a</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>amplificacao_f_sobre_a</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>share_indireto</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>encadeamento_tras_U</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>encadeamento_frente_Uf</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>multiplicador_producao_m</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>intensidade_per_trab_a_tilde</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>pegada_per_trab_f_tilde</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>coef_emprego_e</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>multiplicador_emprego_me</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>quadrante</t>
         </is>
@@ -2922,189 +2910,189 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>codigo</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>0191</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>0192</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>0280</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>0580</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>0680</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>0791</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>1000</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>1300</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>1600</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>1700</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>1900</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>2000</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>2300</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>2400</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>2500</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>2900</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>3500</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>4180</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>4500</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>4900</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>5280</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>5500</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>5800</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>6480</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>6800</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>6900</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>7800</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>8400</t>
         </is>
       </c>
-      <c r="AD1" s="1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>8591</t>
         </is>
       </c>
-      <c r="AE1" s="1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>8592</t>
         </is>
       </c>
-      <c r="AF1" s="1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>8691</t>
         </is>
       </c>
-      <c r="AG1" s="1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t>8692</t>
         </is>
       </c>
-      <c r="AH1" s="1" t="inlineStr">
+      <c r="AH1" t="inlineStr">
         <is>
           <t>9080</t>
         </is>
       </c>
-      <c r="AI1" s="1" t="inlineStr">
+      <c r="AI1" t="inlineStr">
         <is>
           <t>9480</t>
         </is>
       </c>
-      <c r="AJ1" s="1" t="inlineStr">
+      <c r="AJ1" t="inlineStr">
         <is>
           <t>9700</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>0191</t>
         </is>
@@ -3216,7 +3204,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>0192</t>
         </is>
@@ -3328,7 +3316,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>0280</t>
         </is>
@@ -3440,7 +3428,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>0580</t>
         </is>
@@ -3552,7 +3540,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="inlineStr">
+      <c r="A6" t="inlineStr">
         <is>
           <t>0680</t>
         </is>
@@ -3664,7 +3652,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="inlineStr">
+      <c r="A7" t="inlineStr">
         <is>
           <t>0791</t>
         </is>
@@ -3776,7 +3764,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="inlineStr">
+      <c r="A8" t="inlineStr">
         <is>
           <t>1000</t>
         </is>
@@ -3888,7 +3876,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="1" t="inlineStr">
+      <c r="A9" t="inlineStr">
         <is>
           <t>1300</t>
         </is>
@@ -4000,7 +3988,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="1" t="inlineStr">
+      <c r="A10" t="inlineStr">
         <is>
           <t>1600</t>
         </is>
@@ -4112,7 +4100,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="1" t="inlineStr">
+      <c r="A11" t="inlineStr">
         <is>
           <t>1700</t>
         </is>
@@ -4224,7 +4212,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="1" t="inlineStr">
+      <c r="A12" t="inlineStr">
         <is>
           <t>1900</t>
         </is>
@@ -4336,7 +4324,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="1" t="inlineStr">
+      <c r="A13" t="inlineStr">
         <is>
           <t>2000</t>
         </is>
@@ -4448,7 +4436,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="1" t="inlineStr">
+      <c r="A14" t="inlineStr">
         <is>
           <t>2300</t>
         </is>
@@ -4560,7 +4548,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="1" t="inlineStr">
+      <c r="A15" t="inlineStr">
         <is>
           <t>2400</t>
         </is>
@@ -4672,7 +4660,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="1" t="inlineStr">
+      <c r="A16" t="inlineStr">
         <is>
           <t>2500</t>
         </is>
@@ -4784,7 +4772,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="1" t="inlineStr">
+      <c r="A17" t="inlineStr">
         <is>
           <t>2900</t>
         </is>
@@ -4896,7 +4884,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="1" t="inlineStr">
+      <c r="A18" t="inlineStr">
         <is>
           <t>3500</t>
         </is>
@@ -5008,7 +4996,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="1" t="inlineStr">
+      <c r="A19" t="inlineStr">
         <is>
           <t>4180</t>
         </is>
@@ -5120,7 +5108,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="1" t="inlineStr">
+      <c r="A20" t="inlineStr">
         <is>
           <t>4500</t>
         </is>
@@ -5232,7 +5220,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="1" t="inlineStr">
+      <c r="A21" t="inlineStr">
         <is>
           <t>4900</t>
         </is>
@@ -5344,7 +5332,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="1" t="inlineStr">
+      <c r="A22" t="inlineStr">
         <is>
           <t>5280</t>
         </is>
@@ -5456,7 +5444,7 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="1" t="inlineStr">
+      <c r="A23" t="inlineStr">
         <is>
           <t>5500</t>
         </is>
@@ -5568,7 +5556,7 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="1" t="inlineStr">
+      <c r="A24" t="inlineStr">
         <is>
           <t>5800</t>
         </is>
@@ -5680,7 +5668,7 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="1" t="inlineStr">
+      <c r="A25" t="inlineStr">
         <is>
           <t>6480</t>
         </is>
@@ -5792,7 +5780,7 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="1" t="inlineStr">
+      <c r="A26" t="inlineStr">
         <is>
           <t>6800</t>
         </is>
@@ -5904,7 +5892,7 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="1" t="inlineStr">
+      <c r="A27" t="inlineStr">
         <is>
           <t>6900</t>
         </is>
@@ -6016,7 +6004,7 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="1" t="inlineStr">
+      <c r="A28" t="inlineStr">
         <is>
           <t>7800</t>
         </is>
@@ -6128,7 +6116,7 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="1" t="inlineStr">
+      <c r="A29" t="inlineStr">
         <is>
           <t>8400</t>
         </is>
@@ -6240,7 +6228,7 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="1" t="inlineStr">
+      <c r="A30" t="inlineStr">
         <is>
           <t>8591</t>
         </is>
@@ -6352,7 +6340,7 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="1" t="inlineStr">
+      <c r="A31" t="inlineStr">
         <is>
           <t>8592</t>
         </is>
@@ -6464,7 +6452,7 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="1" t="inlineStr">
+      <c r="A32" t="inlineStr">
         <is>
           <t>8691</t>
         </is>
@@ -6576,7 +6564,7 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="1" t="inlineStr">
+      <c r="A33" t="inlineStr">
         <is>
           <t>8692</t>
         </is>
@@ -6688,7 +6676,7 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="1" t="inlineStr">
+      <c r="A34" t="inlineStr">
         <is>
           <t>9080</t>
         </is>
@@ -6800,7 +6788,7 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="1" t="inlineStr">
+      <c r="A35" t="inlineStr">
         <is>
           <t>9480</t>
         </is>
@@ -6912,7 +6900,7 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="1" t="inlineStr">
+      <c r="A36" t="inlineStr">
         <is>
           <t>9700</t>
         </is>
@@ -7038,189 +7026,189 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>codigo</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>0191</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>0192</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>0280</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>0580</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>0680</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>0791</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>1000</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>1300</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>1600</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>1700</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>1900</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>2000</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>2300</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>2400</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>2500</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>2900</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>3500</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>4180</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>4500</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>4900</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>5280</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>5500</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>5800</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>6480</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>6800</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>6900</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>7800</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>8400</t>
         </is>
       </c>
-      <c r="AD1" s="1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>8591</t>
         </is>
       </c>
-      <c r="AE1" s="1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>8592</t>
         </is>
       </c>
-      <c r="AF1" s="1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>8691</t>
         </is>
       </c>
-      <c r="AG1" s="1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t>8692</t>
         </is>
       </c>
-      <c r="AH1" s="1" t="inlineStr">
+      <c r="AH1" t="inlineStr">
         <is>
           <t>9080</t>
         </is>
       </c>
-      <c r="AI1" s="1" t="inlineStr">
+      <c r="AI1" t="inlineStr">
         <is>
           <t>9480</t>
         </is>
       </c>
-      <c r="AJ1" s="1" t="inlineStr">
+      <c r="AJ1" t="inlineStr">
         <is>
           <t>9700</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>0191</t>
         </is>
@@ -7332,7 +7320,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>0192</t>
         </is>
@@ -7444,7 +7432,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>0280</t>
         </is>
@@ -7556,7 +7544,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>0580</t>
         </is>
@@ -7668,7 +7656,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="inlineStr">
+      <c r="A6" t="inlineStr">
         <is>
           <t>0680</t>
         </is>
@@ -7780,7 +7768,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="inlineStr">
+      <c r="A7" t="inlineStr">
         <is>
           <t>0791</t>
         </is>
@@ -7892,7 +7880,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="inlineStr">
+      <c r="A8" t="inlineStr">
         <is>
           <t>1000</t>
         </is>
@@ -8004,7 +7992,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="1" t="inlineStr">
+      <c r="A9" t="inlineStr">
         <is>
           <t>1300</t>
         </is>
@@ -8116,7 +8104,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="1" t="inlineStr">
+      <c r="A10" t="inlineStr">
         <is>
           <t>1600</t>
         </is>
@@ -8228,7 +8216,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="1" t="inlineStr">
+      <c r="A11" t="inlineStr">
         <is>
           <t>1700</t>
         </is>
@@ -8340,7 +8328,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="1" t="inlineStr">
+      <c r="A12" t="inlineStr">
         <is>
           <t>1900</t>
         </is>
@@ -8452,7 +8440,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="1" t="inlineStr">
+      <c r="A13" t="inlineStr">
         <is>
           <t>2000</t>
         </is>
@@ -8564,7 +8552,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="1" t="inlineStr">
+      <c r="A14" t="inlineStr">
         <is>
           <t>2300</t>
         </is>
@@ -8676,7 +8664,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="1" t="inlineStr">
+      <c r="A15" t="inlineStr">
         <is>
           <t>2400</t>
         </is>
@@ -8788,7 +8776,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="1" t="inlineStr">
+      <c r="A16" t="inlineStr">
         <is>
           <t>2500</t>
         </is>
@@ -8900,7 +8888,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="1" t="inlineStr">
+      <c r="A17" t="inlineStr">
         <is>
           <t>2900</t>
         </is>
@@ -9012,7 +9000,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="1" t="inlineStr">
+      <c r="A18" t="inlineStr">
         <is>
           <t>3500</t>
         </is>
@@ -9124,7 +9112,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="1" t="inlineStr">
+      <c r="A19" t="inlineStr">
         <is>
           <t>4180</t>
         </is>
@@ -9236,7 +9224,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="1" t="inlineStr">
+      <c r="A20" t="inlineStr">
         <is>
           <t>4500</t>
         </is>
@@ -9348,7 +9336,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="1" t="inlineStr">
+      <c r="A21" t="inlineStr">
         <is>
           <t>4900</t>
         </is>
@@ -9460,7 +9448,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="1" t="inlineStr">
+      <c r="A22" t="inlineStr">
         <is>
           <t>5280</t>
         </is>
@@ -9572,7 +9560,7 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="1" t="inlineStr">
+      <c r="A23" t="inlineStr">
         <is>
           <t>5500</t>
         </is>
@@ -9684,7 +9672,7 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="1" t="inlineStr">
+      <c r="A24" t="inlineStr">
         <is>
           <t>5800</t>
         </is>
@@ -9796,7 +9784,7 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="1" t="inlineStr">
+      <c r="A25" t="inlineStr">
         <is>
           <t>6480</t>
         </is>
@@ -9908,7 +9896,7 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="1" t="inlineStr">
+      <c r="A26" t="inlineStr">
         <is>
           <t>6800</t>
         </is>
@@ -10020,7 +10008,7 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="1" t="inlineStr">
+      <c r="A27" t="inlineStr">
         <is>
           <t>6900</t>
         </is>
@@ -10132,7 +10120,7 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="1" t="inlineStr">
+      <c r="A28" t="inlineStr">
         <is>
           <t>7800</t>
         </is>
@@ -10244,7 +10232,7 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="1" t="inlineStr">
+      <c r="A29" t="inlineStr">
         <is>
           <t>8400</t>
         </is>
@@ -10356,7 +10344,7 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="1" t="inlineStr">
+      <c r="A30" t="inlineStr">
         <is>
           <t>8591</t>
         </is>
@@ -10468,7 +10456,7 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="1" t="inlineStr">
+      <c r="A31" t="inlineStr">
         <is>
           <t>8592</t>
         </is>
@@ -10580,7 +10568,7 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="1" t="inlineStr">
+      <c r="A32" t="inlineStr">
         <is>
           <t>8691</t>
         </is>
@@ -10692,7 +10680,7 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="1" t="inlineStr">
+      <c r="A33" t="inlineStr">
         <is>
           <t>8692</t>
         </is>
@@ -10804,7 +10792,7 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="1" t="inlineStr">
+      <c r="A34" t="inlineStr">
         <is>
           <t>9080</t>
         </is>
@@ -10916,7 +10904,7 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="1" t="inlineStr">
+      <c r="A35" t="inlineStr">
         <is>
           <t>9480</t>
         </is>
@@ -11028,7 +11016,7 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="1" t="inlineStr">
+      <c r="A36" t="inlineStr">
         <is>
           <t>9700</t>
         </is>
@@ -11154,189 +11142,189 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>codigo</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>0191</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>0192</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>0280</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>0580</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>0680</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>0791</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>1000</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>1300</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>1600</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>1700</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>1900</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>2000</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>2300</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>2400</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>2500</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>2900</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>3500</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>4180</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>4500</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>4900</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>5280</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>5500</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>5800</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>6480</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>6800</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>6900</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>7800</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>8400</t>
         </is>
       </c>
-      <c r="AD1" s="1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>8591</t>
         </is>
       </c>
-      <c r="AE1" s="1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>8592</t>
         </is>
       </c>
-      <c r="AF1" s="1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>8691</t>
         </is>
       </c>
-      <c r="AG1" s="1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t>8692</t>
         </is>
       </c>
-      <c r="AH1" s="1" t="inlineStr">
+      <c r="AH1" t="inlineStr">
         <is>
           <t>9080</t>
         </is>
       </c>
-      <c r="AI1" s="1" t="inlineStr">
+      <c r="AI1" t="inlineStr">
         <is>
           <t>9480</t>
         </is>
       </c>
-      <c r="AJ1" s="1" t="inlineStr">
+      <c r="AJ1" t="inlineStr">
         <is>
           <t>9700</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>0191</t>
         </is>
@@ -11448,7 +11436,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>0192</t>
         </is>
@@ -11560,7 +11548,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>0280</t>
         </is>
@@ -11672,7 +11660,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>0580</t>
         </is>
@@ -11784,7 +11772,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="inlineStr">
+      <c r="A6" t="inlineStr">
         <is>
           <t>0680</t>
         </is>
@@ -11896,7 +11884,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="inlineStr">
+      <c r="A7" t="inlineStr">
         <is>
           <t>0791</t>
         </is>
@@ -12008,7 +11996,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="inlineStr">
+      <c r="A8" t="inlineStr">
         <is>
           <t>1000</t>
         </is>
@@ -12120,7 +12108,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="1" t="inlineStr">
+      <c r="A9" t="inlineStr">
         <is>
           <t>1300</t>
         </is>
@@ -12232,7 +12220,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="1" t="inlineStr">
+      <c r="A10" t="inlineStr">
         <is>
           <t>1600</t>
         </is>
@@ -12344,7 +12332,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="1" t="inlineStr">
+      <c r="A11" t="inlineStr">
         <is>
           <t>1700</t>
         </is>
@@ -12456,7 +12444,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="1" t="inlineStr">
+      <c r="A12" t="inlineStr">
         <is>
           <t>1900</t>
         </is>
@@ -12568,7 +12556,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="1" t="inlineStr">
+      <c r="A13" t="inlineStr">
         <is>
           <t>2000</t>
         </is>
@@ -12680,7 +12668,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="1" t="inlineStr">
+      <c r="A14" t="inlineStr">
         <is>
           <t>2300</t>
         </is>
@@ -12792,7 +12780,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="1" t="inlineStr">
+      <c r="A15" t="inlineStr">
         <is>
           <t>2400</t>
         </is>
@@ -12904,7 +12892,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="1" t="inlineStr">
+      <c r="A16" t="inlineStr">
         <is>
           <t>2500</t>
         </is>
@@ -13016,7 +13004,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="1" t="inlineStr">
+      <c r="A17" t="inlineStr">
         <is>
           <t>2900</t>
         </is>
@@ -13128,7 +13116,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="1" t="inlineStr">
+      <c r="A18" t="inlineStr">
         <is>
           <t>3500</t>
         </is>
@@ -13240,7 +13228,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="1" t="inlineStr">
+      <c r="A19" t="inlineStr">
         <is>
           <t>4180</t>
         </is>
@@ -13352,7 +13340,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="1" t="inlineStr">
+      <c r="A20" t="inlineStr">
         <is>
           <t>4500</t>
         </is>
@@ -13464,7 +13452,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="1" t="inlineStr">
+      <c r="A21" t="inlineStr">
         <is>
           <t>4900</t>
         </is>
@@ -13576,7 +13564,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="1" t="inlineStr">
+      <c r="A22" t="inlineStr">
         <is>
           <t>5280</t>
         </is>
@@ -13688,7 +13676,7 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="1" t="inlineStr">
+      <c r="A23" t="inlineStr">
         <is>
           <t>5500</t>
         </is>
@@ -13800,7 +13788,7 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="1" t="inlineStr">
+      <c r="A24" t="inlineStr">
         <is>
           <t>5800</t>
         </is>
@@ -13912,7 +13900,7 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="1" t="inlineStr">
+      <c r="A25" t="inlineStr">
         <is>
           <t>6480</t>
         </is>
@@ -14024,7 +14012,7 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="1" t="inlineStr">
+      <c r="A26" t="inlineStr">
         <is>
           <t>6800</t>
         </is>
@@ -14136,7 +14124,7 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="1" t="inlineStr">
+      <c r="A27" t="inlineStr">
         <is>
           <t>6900</t>
         </is>
@@ -14248,7 +14236,7 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="1" t="inlineStr">
+      <c r="A28" t="inlineStr">
         <is>
           <t>7800</t>
         </is>
@@ -14360,7 +14348,7 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="1" t="inlineStr">
+      <c r="A29" t="inlineStr">
         <is>
           <t>8400</t>
         </is>
@@ -14472,7 +14460,7 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="1" t="inlineStr">
+      <c r="A30" t="inlineStr">
         <is>
           <t>8591</t>
         </is>
@@ -14584,7 +14572,7 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="1" t="inlineStr">
+      <c r="A31" t="inlineStr">
         <is>
           <t>8592</t>
         </is>
@@ -14696,7 +14684,7 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="1" t="inlineStr">
+      <c r="A32" t="inlineStr">
         <is>
           <t>8691</t>
         </is>
@@ -14808,7 +14796,7 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="1" t="inlineStr">
+      <c r="A33" t="inlineStr">
         <is>
           <t>8692</t>
         </is>
@@ -14920,7 +14908,7 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="1" t="inlineStr">
+      <c r="A34" t="inlineStr">
         <is>
           <t>9080</t>
         </is>
@@ -15032,7 +15020,7 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="1" t="inlineStr">
+      <c r="A35" t="inlineStr">
         <is>
           <t>9480</t>
         </is>
@@ -15144,7 +15132,7 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="1" t="inlineStr">
+      <c r="A36" t="inlineStr">
         <is>
           <t>9700</t>
         </is>

</xml_diff>